<commit_message>
data: update 2026-09-01 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/daily_logs/daily_2026-09-01.xlsx
+++ b/daily_logs/daily_2026-09-01.xlsx
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>3</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.42</v>
+        <v>2.44</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.73</v>
+        <v>4.75</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>2</v>
+        <v>-5</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.22</v>
+        <v>5.25</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>5</v>
+        <v>-2</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.31</v>
+        <v>2.35</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-4</v>
+        <v>-12</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.31</v>
+        <v>2.33</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.65</v>
+        <v>3.68</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=25.0bp [TRIGGERED]
-HY OAS 5dd=10.0bp
+          <t>HY OAS 20dd=15.0bp [OK]
+HY OAS 5dd=6.0bp
 HYG 5d=0.1% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=-0.4% [OK]

</xml_diff>